<commit_message>
Update Trading Journal.xlsx 2026-09-15 09:57:58
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2195,6 +2195,39 @@
       </c>
       <c r="H49" s="1" t="inlineStr"/>
       <c r="I49" s="1" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>6226</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>光鼎</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr">
+        <is>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr"/>
+      <c r="H50" s="1" t="inlineStr"/>
+      <c r="I50" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-15 09:59:21
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2225,9 +2225,46 @@
           <t>停利賣出</t>
         </is>
       </c>
-      <c r="G50" s="1" t="inlineStr"/>
+      <c r="G50" s="1" t="n">
+        <v>4</v>
+      </c>
       <c r="H50" s="1" t="inlineStr"/>
       <c r="I50" s="1" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>6226</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>光鼎</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="n">
+        <v>32.25</v>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>3K反轉</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H51" s="1" t="inlineStr"/>
+      <c r="I51" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-17 09:27:32
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2261,10 +2261,80 @@
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H51" s="1" t="inlineStr"/>
       <c r="I51" s="1" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>2426</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>鼎元</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="n">
+        <v>92.7</v>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" s="1" t="inlineStr"/>
+      <c r="I52" s="1" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>2426</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>鼎元</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>3K反轉</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" s="1" t="inlineStr"/>
+      <c r="I53" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-17 10:34:13
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2335,6 +2335,41 @@
       </c>
       <c r="H53" s="1" t="inlineStr"/>
       <c r="I53" s="1" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>6168</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>宏齊</t>
+        </is>
+      </c>
+      <c r="D54" s="1" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>下降趨勢線突破</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="H54" s="1" t="inlineStr"/>
+      <c r="I54" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-22 13:11:10
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2370,6 +2370,111 @@
       </c>
       <c r="H54" s="1" t="inlineStr"/>
       <c r="I54" s="1" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>2426</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>鼎元</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="n">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H55" s="1" t="inlineStr"/>
+      <c r="I55" s="1" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="inlineStr">
+        <is>
+          <t>2308</t>
+        </is>
+      </c>
+      <c r="C56" s="1" t="inlineStr">
+        <is>
+          <t>台達電</t>
+        </is>
+      </c>
+      <c r="D56" s="1" t="n">
+        <v>1860</v>
+      </c>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F56" s="1" t="inlineStr">
+        <is>
+          <t>下降趨勢線突破</t>
+        </is>
+      </c>
+      <c r="G56" s="1" t="inlineStr"/>
+      <c r="H56" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="I56" s="1" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>6510</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>精測</t>
+        </is>
+      </c>
+      <c r="D57" s="1" t="n">
+        <v>3725</v>
+      </c>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F57" s="1" t="inlineStr">
+        <is>
+          <t>KD高腳</t>
+        </is>
+      </c>
+      <c r="G57" s="1" t="inlineStr"/>
+      <c r="H57" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I57" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-23 10:15:09
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2475,6 +2475,41 @@
         <v>20</v>
       </c>
       <c r="I57" s="1" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>3081</t>
+        </is>
+      </c>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t>聯亞</t>
+        </is>
+      </c>
+      <c r="D58" s="1" t="n">
+        <v>2610</v>
+      </c>
+      <c r="E58" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F58" s="1" t="inlineStr">
+        <is>
+          <t>停損賣出</t>
+        </is>
+      </c>
+      <c r="G58" s="1" t="inlineStr"/>
+      <c r="H58" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I58" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-29 10:25:04
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2510,6 +2510,177 @@
         <v>100</v>
       </c>
       <c r="I58" s="1" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t>8064</t>
+        </is>
+      </c>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>東捷</t>
+        </is>
+      </c>
+      <c r="D59" s="1" t="n">
+        <v>134</v>
+      </c>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F59" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G59" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" s="1" t="inlineStr"/>
+      <c r="I59" s="1" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B60" s="1" t="inlineStr">
+        <is>
+          <t>8064</t>
+        </is>
+      </c>
+      <c r="C60" s="1" t="inlineStr">
+        <is>
+          <t>東捷</t>
+        </is>
+      </c>
+      <c r="D60" s="1" t="n">
+        <v>137.5</v>
+      </c>
+      <c r="E60" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F60" s="1" t="inlineStr">
+        <is>
+          <t>23戰法買</t>
+        </is>
+      </c>
+      <c r="G60" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" s="1" t="inlineStr"/>
+      <c r="I60" s="1" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>6147</t>
+        </is>
+      </c>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>頎邦</t>
+        </is>
+      </c>
+      <c r="D61" s="1" t="n">
+        <v>211</v>
+      </c>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F61" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G61" s="1" t="inlineStr"/>
+      <c r="H61" s="1" t="inlineStr"/>
+      <c r="I61" s="1" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>4772</t>
+        </is>
+      </c>
+      <c r="C62" s="1" t="inlineStr">
+        <is>
+          <t>台特化</t>
+        </is>
+      </c>
+      <c r="D62" s="1" t="n">
+        <v>268</v>
+      </c>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F62" s="1" t="inlineStr">
+        <is>
+          <t>島狀反轉</t>
+        </is>
+      </c>
+      <c r="G62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" s="1" t="inlineStr"/>
+      <c r="I62" s="1" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t>6588</t>
+        </is>
+      </c>
+      <c r="C63" s="1" t="inlineStr">
+        <is>
+          <t>東典光電</t>
+        </is>
+      </c>
+      <c r="D63" s="1" t="n">
+        <v>110</v>
+      </c>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F63" s="1" t="inlineStr">
+        <is>
+          <t>停損賣出</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="inlineStr"/>
+      <c r="H63" s="1" t="inlineStr"/>
+      <c r="I63" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-29 10:58:29
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2610,7 +2610,9 @@
           <t>巧妙點</t>
         </is>
       </c>
-      <c r="G61" s="1" t="inlineStr"/>
+      <c r="G61" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="H61" s="1" t="inlineStr"/>
       <c r="I61" s="1" t="inlineStr"/>
     </row>
@@ -2678,9 +2680,46 @@
           <t>停損賣出</t>
         </is>
       </c>
-      <c r="G63" s="1" t="inlineStr"/>
+      <c r="G63" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="H63" s="1" t="inlineStr"/>
       <c r="I63" s="1" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B64" s="1" t="inlineStr">
+        <is>
+          <t>6510</t>
+        </is>
+      </c>
+      <c r="C64" s="1" t="inlineStr">
+        <is>
+          <t>精測</t>
+        </is>
+      </c>
+      <c r="D64" s="1" t="n">
+        <v>3155</v>
+      </c>
+      <c r="E64" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F64" s="1" t="inlineStr">
+        <is>
+          <t>停損賣出</t>
+        </is>
+      </c>
+      <c r="G64" s="1" t="inlineStr"/>
+      <c r="H64" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I64" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>